<commit_message>
Recupération des groupes dans les SAE
</commit_message>
<xml_diff>
--- a/GestionServiceGeii-WPF/TestData/GEII_selection_reference.xlsx
+++ b/GestionServiceGeii-WPF/TestData/GEII_selection_reference.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e6ac49f9f1cc6e68/@33 - VS_PRO_2026/source/repos/GestionServiceGeii-WPF/GestionServiceGeii-WPF/TestData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="366" documentId="8_{4DFBFF07-CFCD-44D6-8C2F-9787859927BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3751F7C3-061C-4563-8277-7C4118D37886}"/>
+  <xr:revisionPtr revIDLastSave="383" documentId="8_{4DFBFF07-CFCD-44D6-8C2F-9787859927BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48DC556E-1DD1-4E31-9319-61D0219502B4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7687" uniqueCount="741">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7687" uniqueCount="742">
   <si>
     <t>Formation</t>
   </si>
@@ -2240,12 +2240,6 @@
     <t>R3-ESE-15</t>
   </si>
   <si>
-    <t>S3-ESE-1</t>
-  </si>
-  <si>
-    <t>S3-ESE-2</t>
-  </si>
-  <si>
     <t>R3-EME-13</t>
   </si>
   <si>
@@ -2258,9 +2252,6 @@
     <t>R3-EME-16</t>
   </si>
   <si>
-    <t>S3-EME-1</t>
-  </si>
-  <si>
     <t>R3-AII-13</t>
   </si>
   <si>
@@ -2273,13 +2264,25 @@
     <t>R3-AII-16</t>
   </si>
   <si>
-    <t>S3-AII-1</t>
-  </si>
-  <si>
-    <t>S3-AII-2</t>
-  </si>
-  <si>
     <t>R3-EME-12</t>
+  </si>
+  <si>
+    <t>SAE31-ESE</t>
+  </si>
+  <si>
+    <t>SAE31-EME</t>
+  </si>
+  <si>
+    <t>SAE31-AII</t>
+  </si>
+  <si>
+    <t>SAE32-ESE</t>
+  </si>
+  <si>
+    <t>SAE32-EME</t>
+  </si>
+  <si>
+    <t>SAE32-AII</t>
   </si>
 </sst>
 </file>
@@ -11861,7 +11864,7 @@
         <v>109</v>
       </c>
       <c r="F54" t="s">
-        <v>727</v>
+        <v>736</v>
       </c>
       <c r="G54" s="31">
         <v>0</v>
@@ -11890,7 +11893,7 @@
         <v>111</v>
       </c>
       <c r="F55" s="101" t="s">
-        <v>728</v>
+        <v>739</v>
       </c>
       <c r="G55" s="108">
         <v>0</v>
@@ -11919,7 +11922,7 @@
         <v>289</v>
       </c>
       <c r="F56" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="G56" s="106">
         <v>3</v>
@@ -11948,7 +11951,7 @@
         <v>290</v>
       </c>
       <c r="F57" t="s">
-        <v>730</v>
+        <v>728</v>
       </c>
       <c r="G57" s="106">
         <v>0</v>
@@ -11977,7 +11980,7 @@
         <v>113</v>
       </c>
       <c r="F58" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="G58" s="110">
         <v>0</v>
@@ -12006,7 +12009,7 @@
         <v>115</v>
       </c>
       <c r="F59" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="G59" s="110">
         <v>0</v>
@@ -12035,7 +12038,7 @@
         <v>115</v>
       </c>
       <c r="F60" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="G60" s="31">
         <v>0</v>
@@ -12064,7 +12067,7 @@
         <v>291</v>
       </c>
       <c r="F61" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="G61" s="31">
         <v>0</v>
@@ -12090,10 +12093,10 @@
         <v>110</v>
       </c>
       <c r="E62" s="101" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F62" s="101" t="s">
-        <v>733</v>
+        <v>740</v>
       </c>
       <c r="G62" s="108">
         <v>0</v>
@@ -12122,7 +12125,7 @@
         <v>710</v>
       </c>
       <c r="F63" t="s">
-        <v>734</v>
+        <v>731</v>
       </c>
       <c r="G63" s="110">
         <v>0</v>
@@ -12151,7 +12154,7 @@
         <v>293</v>
       </c>
       <c r="F64" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="G64" s="110">
         <v>0</v>
@@ -12180,7 +12183,7 @@
         <v>294</v>
       </c>
       <c r="F65" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="G65" s="110">
         <v>0</v>
@@ -12209,7 +12212,7 @@
         <v>119</v>
       </c>
       <c r="F66" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="G66" s="110">
         <v>0</v>
@@ -12267,7 +12270,7 @@
         <v>295</v>
       </c>
       <c r="F68" s="101" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="G68" s="114">
         <v>0</v>
@@ -12673,7 +12676,7 @@
         <v>159</v>
       </c>
       <c r="F82" t="s">
-        <v>740</v>
+        <v>735</v>
       </c>
       <c r="G82" s="110">
         <v>0</v>
@@ -12702,7 +12705,7 @@
         <v>113</v>
       </c>
       <c r="F83" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="G83" s="110">
         <v>0</v>
@@ -12731,7 +12734,7 @@
         <v>115</v>
       </c>
       <c r="F84" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="G84" s="110">
         <v>0</v>
@@ -12760,7 +12763,7 @@
         <v>113</v>
       </c>
       <c r="F85" t="s">
-        <v>731</v>
+        <v>729</v>
       </c>
       <c r="G85" s="110">
         <v>0</v>
@@ -12818,7 +12821,7 @@
         <v>115</v>
       </c>
       <c r="F87" t="s">
-        <v>732</v>
+        <v>730</v>
       </c>
       <c r="G87" s="110">
         <v>0</v>
@@ -12905,7 +12908,7 @@
         <v>294</v>
       </c>
       <c r="F90" t="s">
-        <v>736</v>
+        <v>733</v>
       </c>
       <c r="G90" s="110">
         <v>0</v>
@@ -12934,7 +12937,7 @@
         <v>119</v>
       </c>
       <c r="F91" t="s">
-        <v>737</v>
+        <v>734</v>
       </c>
       <c r="G91" s="110">
         <v>0</v>
@@ -12963,7 +12966,7 @@
         <v>109</v>
       </c>
       <c r="F92" t="s">
-        <v>727</v>
+        <v>736</v>
       </c>
       <c r="G92" s="110">
         <v>0</v>
@@ -12992,7 +12995,7 @@
         <v>291</v>
       </c>
       <c r="F93" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="G93" s="110">
         <v>0</v>

</xml_diff>

<commit_message>
Point de repère S4 avant retour sur S1 S2
</commit_message>
<xml_diff>
--- a/GestionServiceGeii-WPF/TestData/GEII_selection_reference.xlsx
+++ b/GestionServiceGeii-WPF/TestData/GEII_selection_reference.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e6ac49f9f1cc6e68/@33 - VS_PRO_2026/source/repos/GestionServiceGeii-WPF/GestionServiceGeii-WPF/TestData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="590" documentId="8_{4DFBFF07-CFCD-44D6-8C2F-9787859927BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4A71B9E-F23D-452D-A962-EFEAAA7A879C}"/>
+  <xr:revisionPtr revIDLastSave="598" documentId="8_{4DFBFF07-CFCD-44D6-8C2F-9787859927BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{83F1E756-5716-402D-BC96-FD63A5F1E63D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UE" sheetId="1" r:id="rId1"/>
@@ -2830,7 +2830,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="125">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3071,10 +3071,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3087,9 +3084,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3119,11 +3113,6 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3135,6 +3124,27 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79992065187536243"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="0.79992065187536243"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3183,27 +3193,6 @@
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.79992065187536243"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="0.79992065187536243"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3217,12 +3206,15 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4B8BFAE3-6CEA-40E4-8F60-C9E9BDB42CB9}" name="TableauModule" displayName="TableauModule" ref="A1:J139" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4B8BFAE3-6CEA-40E4-8F60-C9E9BDB42CB9}" name="TableauModule" displayName="TableauModule" ref="A1:J139" totalsRowShown="0" headerRowDxfId="7">
   <autoFilter ref="A1:J139" xr:uid="{4B8BFAE3-6CEA-40E4-8F60-C9E9BDB42CB9}">
     <filterColumn colId="0">
       <filters>
-        <filter val="S3"/>
         <filter val="S4"/>
       </filters>
     </filterColumn>
@@ -3234,10 +3226,10 @@
     <tableColumn id="4" xr3:uid="{667903B8-7DE7-4AB0-95E2-7B0111443166}" name="MODULE"/>
     <tableColumn id="5" xr3:uid="{FFAC88E5-6BAC-432B-986D-1B7EFEBEAC75}" name="OSE"/>
     <tableColumn id="9" xr3:uid="{0931D180-C889-4F8A-A9B6-F3A2A40736C6}" name="CodePedagogique"/>
-    <tableColumn id="6" xr3:uid="{83D20F3C-F050-4307-AC62-E170BED4C879}" name="CM" dataDxfId="3"/>
-    <tableColumn id="10" xr3:uid="{8095D425-FCB0-41D5-8848-364A7822EAB4}" name="APP" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{9E43D79F-998B-480D-84DE-E6C9F0C1BF70}" name="TD" dataDxfId="1"/>
-    <tableColumn id="8" xr3:uid="{943F5095-89DA-4E6D-9A3A-58C9EA05739F}" name="TP" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{83D20F3C-F050-4307-AC62-E170BED4C879}" name="CM" dataDxfId="6"/>
+    <tableColumn id="10" xr3:uid="{8095D425-FCB0-41D5-8848-364A7822EAB4}" name="APP" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{9E43D79F-998B-480D-84DE-E6C9F0C1BF70}" name="TD" dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{943F5095-89DA-4E6D-9A3A-58C9EA05739F}" name="TP" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3250,8 +3242,8 @@
     <sortCondition ref="A1:A29"/>
   </sortState>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{CC4027AC-8F91-4B5F-98D6-BF1E296EE67E}" name="Titulaires" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{A272B22C-7A7F-43DD-9DF7-144DFBDCD668}" name="Prenom" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{CC4027AC-8F91-4B5F-98D6-BF1E296EE67E}" name="Titulaires" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{A272B22C-7A7F-43DD-9DF7-144DFBDCD668}" name="Prenom" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{38AE9C4C-9A4D-498C-871D-A3F993D7DD43}" name="Statut"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -3262,7 +3254,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{066A705B-E44A-4479-B699-F7F7B3AAE3B0}" name="Tableau3" displayName="Tableau3" ref="A1:C34" totalsRowShown="0">
   <autoFilter ref="A1:C34" xr:uid="{066A705B-E44A-4479-B699-F7F7B3AAE3B0}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{45F2EF42-A849-4931-8857-D315F7A529A5}" name="Vacataires" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{45F2EF42-A849-4931-8857-D315F7A529A5}" name="Vacataires" dataDxfId="0"/>
     <tableColumn id="2" xr3:uid="{F64808F6-8546-4B29-ACC4-26ABE465BFB0}" name="Prenom"/>
     <tableColumn id="3" xr3:uid="{46505AF3-08EF-482B-93D4-E17DBF509EED}" name="Statut"/>
   </tableColumns>
@@ -8127,12 +8119,12 @@
       </c>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" s="123" t="s">
+      <c r="A4" s="118" t="s">
         <v>761</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="124" t="s">
+      <c r="A5" s="119" t="s">
         <v>762</v>
       </c>
     </row>
@@ -8797,14 +8789,14 @@
         <v>50</v>
       </c>
       <c r="F19" s="88"/>
-      <c r="G19" s="104">
+      <c r="G19" s="103">
         <v>0</v>
       </c>
-      <c r="H19" s="104"/>
-      <c r="I19" s="104">
+      <c r="H19" s="103"/>
+      <c r="I19" s="103">
         <v>10</v>
       </c>
-      <c r="J19" s="105">
+      <c r="J19" s="104">
         <v>16</v>
       </c>
       <c r="L19" s="88"/>
@@ -9285,18 +9277,18 @@
         <v>66</v>
       </c>
       <c r="F37" s="88"/>
-      <c r="G37" s="104">
+      <c r="G37" s="103">
         <v>0</v>
       </c>
-      <c r="H37" s="104"/>
-      <c r="I37" s="104">
+      <c r="H37" s="103"/>
+      <c r="I37" s="103">
         <v>10</v>
       </c>
-      <c r="J37" s="105">
+      <c r="J37" s="104">
         <v>16</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" hidden="1">
       <c r="A38" t="s">
         <v>6</v>
       </c>
@@ -9328,7 +9320,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" hidden="1">
       <c r="A39" t="s">
         <v>6</v>
       </c>
@@ -9360,7 +9352,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
+    <row r="40" spans="1:10" hidden="1">
       <c r="A40" t="s">
         <v>6</v>
       </c>
@@ -9392,7 +9384,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:10">
+    <row r="41" spans="1:10" hidden="1">
       <c r="A41" t="s">
         <v>6</v>
       </c>
@@ -9424,7 +9416,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:10">
+    <row r="42" spans="1:10" hidden="1">
       <c r="A42" t="s">
         <v>6</v>
       </c>
@@ -9456,7 +9448,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="43" spans="1:10">
+    <row r="43" spans="1:10" hidden="1">
       <c r="A43" t="s">
         <v>6</v>
       </c>
@@ -9488,7 +9480,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:10">
+    <row r="44" spans="1:10" hidden="1">
       <c r="A44" t="s">
         <v>6</v>
       </c>
@@ -9520,7 +9512,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="1:10">
+    <row r="45" spans="1:10" hidden="1">
       <c r="A45" t="s">
         <v>6</v>
       </c>
@@ -9552,7 +9544,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="46" spans="1:10">
+    <row r="46" spans="1:10" hidden="1">
       <c r="A46" t="s">
         <v>6</v>
       </c>
@@ -9584,7 +9576,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:10">
+    <row r="47" spans="1:10" hidden="1">
       <c r="A47" t="s">
         <v>6</v>
       </c>
@@ -9616,7 +9608,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="48" spans="1:10">
+    <row r="48" spans="1:10" hidden="1">
       <c r="A48" t="s">
         <v>6</v>
       </c>
@@ -9648,7 +9640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:10">
+    <row r="49" spans="1:10" hidden="1">
       <c r="A49" s="88" t="s">
         <v>6</v>
       </c>
@@ -9670,7 +9662,7 @@
       <c r="G49" s="99">
         <v>1</v>
       </c>
-      <c r="H49" s="116">
+      <c r="H49" s="114">
         <v>1</v>
       </c>
       <c r="I49" s="99">
@@ -9680,7 +9672,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:10">
+    <row r="50" spans="1:10" hidden="1">
       <c r="A50" t="s">
         <v>6</v>
       </c>
@@ -9699,20 +9691,20 @@
       <c r="F50" t="s">
         <v>120</v>
       </c>
-      <c r="G50" s="106">
+      <c r="G50" s="105">
         <v>3</v>
       </c>
       <c r="H50" s="89">
         <v>3</v>
       </c>
-      <c r="I50" s="106">
+      <c r="I50" s="105">
         <v>26</v>
       </c>
-      <c r="J50" s="107">
+      <c r="J50" s="106">
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:10">
+    <row r="51" spans="1:10" hidden="1">
       <c r="A51" t="s">
         <v>6</v>
       </c>
@@ -9731,20 +9723,20 @@
       <c r="F51" t="s">
         <v>122</v>
       </c>
-      <c r="G51" s="106">
+      <c r="G51" s="105">
         <v>0</v>
       </c>
       <c r="H51" s="89">
         <v>0</v>
       </c>
-      <c r="I51" s="106">
+      <c r="I51" s="105">
         <v>8</v>
       </c>
-      <c r="J51" s="107">
+      <c r="J51" s="106">
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="1:10">
+    <row r="52" spans="1:10" hidden="1">
       <c r="A52" t="s">
         <v>6</v>
       </c>
@@ -9763,20 +9755,20 @@
       <c r="F52" t="s">
         <v>124</v>
       </c>
-      <c r="G52" s="108">
+      <c r="G52" s="102">
         <v>0</v>
       </c>
       <c r="H52" s="89">
         <v>0</v>
       </c>
-      <c r="I52" s="108">
+      <c r="I52" s="102">
         <v>12</v>
       </c>
-      <c r="J52" s="109">
+      <c r="J52" s="107">
         <v>18</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
+    <row r="53" spans="1:10" hidden="1">
       <c r="A53" t="s">
         <v>6</v>
       </c>
@@ -9795,20 +9787,20 @@
       <c r="F53" t="s">
         <v>124</v>
       </c>
-      <c r="G53" s="108">
+      <c r="G53" s="102">
         <v>0</v>
       </c>
       <c r="H53" s="89">
         <v>0</v>
       </c>
-      <c r="I53" s="108">
+      <c r="I53" s="102">
         <v>12</v>
       </c>
-      <c r="J53" s="109">
+      <c r="J53" s="107">
         <v>12</v>
       </c>
     </row>
-    <row r="54" spans="1:10">
+    <row r="54" spans="1:10" hidden="1">
       <c r="A54" t="s">
         <v>6</v>
       </c>
@@ -9840,7 +9832,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="55" spans="1:10">
+    <row r="55" spans="1:10" hidden="1">
       <c r="A55" s="88" t="s">
         <v>6</v>
       </c>
@@ -9859,20 +9851,20 @@
       <c r="F55" s="88" t="s">
         <v>131</v>
       </c>
-      <c r="G55" s="110">
+      <c r="G55" s="108">
         <v>0</v>
       </c>
-      <c r="H55" s="116">
+      <c r="H55" s="114">
         <v>0</v>
       </c>
-      <c r="I55" s="110">
+      <c r="I55" s="108">
         <v>0</v>
       </c>
-      <c r="J55" s="111">
+      <c r="J55" s="109">
         <v>32</v>
       </c>
     </row>
-    <row r="56" spans="1:10">
+    <row r="56" spans="1:10" hidden="1">
       <c r="A56" t="s">
         <v>6</v>
       </c>
@@ -9891,20 +9883,20 @@
       <c r="F56" t="s">
         <v>134</v>
       </c>
-      <c r="G56" s="106">
+      <c r="G56" s="105">
         <v>3</v>
       </c>
       <c r="H56" s="89">
         <v>3</v>
       </c>
-      <c r="I56" s="106">
+      <c r="I56" s="105">
         <v>26</v>
       </c>
-      <c r="J56" s="107">
+      <c r="J56" s="106">
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:10">
+    <row r="57" spans="1:10" hidden="1">
       <c r="A57" t="s">
         <v>6</v>
       </c>
@@ -9923,20 +9915,20 @@
       <c r="F57" t="s">
         <v>136</v>
       </c>
-      <c r="G57" s="106">
+      <c r="G57" s="105">
         <v>0</v>
       </c>
       <c r="H57" s="89">
         <v>0</v>
       </c>
-      <c r="I57" s="106">
+      <c r="I57" s="105">
         <v>8</v>
       </c>
-      <c r="J57" s="107">
+      <c r="J57" s="106">
         <v>16</v>
       </c>
     </row>
-    <row r="58" spans="1:10">
+    <row r="58" spans="1:10" hidden="1">
       <c r="A58" t="s">
         <v>6</v>
       </c>
@@ -9955,20 +9947,20 @@
       <c r="F58" t="s">
         <v>139</v>
       </c>
-      <c r="G58" s="108">
+      <c r="G58" s="102">
         <v>0</v>
       </c>
       <c r="H58" s="89">
         <v>0</v>
       </c>
-      <c r="I58" s="108">
+      <c r="I58" s="102">
         <v>10</v>
       </c>
-      <c r="J58" s="109">
+      <c r="J58" s="107">
         <v>16</v>
       </c>
     </row>
-    <row r="59" spans="1:10">
+    <row r="59" spans="1:10" hidden="1">
       <c r="A59" t="s">
         <v>6</v>
       </c>
@@ -9987,20 +9979,20 @@
       <c r="F59" t="s">
         <v>142</v>
       </c>
-      <c r="G59" s="108">
+      <c r="G59" s="102">
         <v>0</v>
       </c>
       <c r="H59" s="89">
         <v>0</v>
       </c>
-      <c r="I59" s="108">
+      <c r="I59" s="102">
         <v>12</v>
       </c>
-      <c r="J59" s="109">
+      <c r="J59" s="107">
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="1:10">
+    <row r="60" spans="1:10" hidden="1">
       <c r="A60" t="s">
         <v>6</v>
       </c>
@@ -10032,7 +10024,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="61" spans="1:10">
+    <row r="61" spans="1:10" hidden="1">
       <c r="A61" t="s">
         <v>6</v>
       </c>
@@ -10064,7 +10056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:10">
+    <row r="62" spans="1:10" hidden="1">
       <c r="A62" s="88" t="s">
         <v>6</v>
       </c>
@@ -10083,20 +10075,20 @@
       <c r="F62" s="88" t="s">
         <v>147</v>
       </c>
-      <c r="G62" s="110">
+      <c r="G62" s="108">
         <v>0</v>
       </c>
-      <c r="H62" s="116">
+      <c r="H62" s="114">
         <v>0</v>
       </c>
-      <c r="I62" s="110">
+      <c r="I62" s="108">
         <v>0</v>
       </c>
-      <c r="J62" s="111">
+      <c r="J62" s="109">
         <v>32</v>
       </c>
     </row>
-    <row r="63" spans="1:10">
+    <row r="63" spans="1:10" hidden="1">
       <c r="A63" t="s">
         <v>6</v>
       </c>
@@ -10115,20 +10107,20 @@
       <c r="F63" t="s">
         <v>150</v>
       </c>
-      <c r="G63" s="108">
+      <c r="G63" s="102">
         <v>0</v>
       </c>
       <c r="H63" s="89">
         <v>0</v>
       </c>
-      <c r="I63" s="108">
+      <c r="I63" s="102">
         <v>0</v>
       </c>
-      <c r="J63" s="109">
+      <c r="J63" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:10">
+    <row r="64" spans="1:10" hidden="1">
       <c r="A64" t="s">
         <v>6</v>
       </c>
@@ -10147,20 +10139,20 @@
       <c r="F64" t="s">
         <v>152</v>
       </c>
-      <c r="G64" s="108">
+      <c r="G64" s="102">
         <v>0</v>
       </c>
       <c r="H64" s="89">
         <v>0</v>
       </c>
-      <c r="I64" s="108">
+      <c r="I64" s="102">
         <v>0</v>
       </c>
-      <c r="J64" s="109">
+      <c r="J64" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:10" hidden="1">
       <c r="A65" t="s">
         <v>6</v>
       </c>
@@ -10179,20 +10171,20 @@
       <c r="F65" t="s">
         <v>154</v>
       </c>
-      <c r="G65" s="108">
+      <c r="G65" s="102">
         <v>0</v>
       </c>
       <c r="H65" s="89">
         <v>0</v>
       </c>
-      <c r="I65" s="108">
+      <c r="I65" s="102">
         <v>0</v>
       </c>
-      <c r="J65" s="109">
+      <c r="J65" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
+    <row r="66" spans="1:10" hidden="1">
       <c r="A66" t="s">
         <v>6</v>
       </c>
@@ -10211,20 +10203,20 @@
       <c r="F66" t="s">
         <v>157</v>
       </c>
-      <c r="G66" s="108">
+      <c r="G66" s="102">
         <v>0</v>
       </c>
       <c r="H66" s="89">
         <v>0</v>
       </c>
-      <c r="I66" s="108">
+      <c r="I66" s="102">
         <v>0</v>
       </c>
-      <c r="J66" s="109">
+      <c r="J66" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:10">
+    <row r="67" spans="1:10" hidden="1">
       <c r="A67" t="s">
         <v>6</v>
       </c>
@@ -10243,20 +10235,20 @@
       <c r="F67" t="s">
         <v>159</v>
       </c>
-      <c r="G67" s="108">
+      <c r="G67" s="102">
         <v>0</v>
       </c>
       <c r="H67" s="89">
         <v>0</v>
       </c>
-      <c r="I67" s="108">
+      <c r="I67" s="102">
         <v>0</v>
       </c>
-      <c r="J67" s="109">
+      <c r="J67" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:10">
+    <row r="68" spans="1:10" hidden="1">
       <c r="A68" s="88" t="s">
         <v>6</v>
       </c>
@@ -10275,20 +10267,20 @@
       <c r="F68" s="88" t="s">
         <v>161</v>
       </c>
-      <c r="G68" s="112">
+      <c r="G68" s="110">
         <v>0</v>
       </c>
-      <c r="H68" s="116">
+      <c r="H68" s="114">
         <v>0</v>
       </c>
-      <c r="I68" s="112">
+      <c r="I68" s="110">
         <v>0</v>
       </c>
-      <c r="J68" s="113">
+      <c r="J68" s="111">
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:10">
+    <row r="69" spans="1:10" hidden="1">
       <c r="A69" t="s">
         <v>6</v>
       </c>
@@ -10307,20 +10299,20 @@
       <c r="F69" t="s">
         <v>84</v>
       </c>
-      <c r="G69" s="108">
+      <c r="G69" s="102">
         <v>0</v>
       </c>
       <c r="H69" s="89">
         <v>0</v>
       </c>
-      <c r="I69" s="108">
+      <c r="I69" s="102">
         <v>10</v>
       </c>
-      <c r="J69" s="109">
+      <c r="J69" s="107">
         <v>12</v>
       </c>
     </row>
-    <row r="70" spans="1:10">
+    <row r="70" spans="1:10" hidden="1">
       <c r="A70" t="s">
         <v>6</v>
       </c>
@@ -10339,20 +10331,20 @@
       <c r="F70" t="s">
         <v>87</v>
       </c>
-      <c r="G70" s="108">
+      <c r="G70" s="102">
         <v>0</v>
       </c>
       <c r="H70" s="89">
         <v>0</v>
       </c>
-      <c r="I70" s="108">
+      <c r="I70" s="102">
         <v>12</v>
       </c>
-      <c r="J70" s="109">
+      <c r="J70" s="107">
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="1:10">
+    <row r="71" spans="1:10" hidden="1">
       <c r="A71" t="s">
         <v>6</v>
       </c>
@@ -10371,20 +10363,20 @@
       <c r="F71" t="s">
         <v>93</v>
       </c>
-      <c r="G71" s="108">
+      <c r="G71" s="102">
         <v>0</v>
       </c>
       <c r="H71" s="89">
         <v>0</v>
       </c>
-      <c r="I71" s="108">
+      <c r="I71" s="102">
         <v>18</v>
       </c>
-      <c r="J71" s="109">
+      <c r="J71" s="107">
         <v>10</v>
       </c>
     </row>
-    <row r="72" spans="1:10">
+    <row r="72" spans="1:10" hidden="1">
       <c r="A72" t="s">
         <v>6</v>
       </c>
@@ -10403,20 +10395,20 @@
       <c r="F72" t="s">
         <v>90</v>
       </c>
-      <c r="G72" s="108">
+      <c r="G72" s="102">
         <v>0</v>
       </c>
       <c r="H72" s="89">
         <v>0</v>
       </c>
-      <c r="I72" s="108">
+      <c r="I72" s="102">
         <v>22</v>
       </c>
-      <c r="J72" s="109">
+      <c r="J72" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:10">
+    <row r="73" spans="1:10" hidden="1">
       <c r="A73" t="s">
         <v>6</v>
       </c>
@@ -10435,20 +10427,20 @@
       <c r="F73" t="s">
         <v>96</v>
       </c>
-      <c r="G73" s="108">
+      <c r="G73" s="102">
         <v>0</v>
       </c>
       <c r="H73" s="89">
         <v>0</v>
       </c>
-      <c r="I73" s="108">
+      <c r="I73" s="102">
         <v>0</v>
       </c>
-      <c r="J73" s="109">
+      <c r="J73" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:10">
+    <row r="74" spans="1:10" hidden="1">
       <c r="A74" t="s">
         <v>6</v>
       </c>
@@ -10467,20 +10459,20 @@
       <c r="F74" t="s">
         <v>99</v>
       </c>
-      <c r="G74" s="108">
+      <c r="G74" s="102">
         <v>0</v>
       </c>
       <c r="H74" s="89">
         <v>0</v>
       </c>
-      <c r="I74" s="108">
+      <c r="I74" s="102">
         <v>0</v>
       </c>
-      <c r="J74" s="109">
+      <c r="J74" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:10">
+    <row r="75" spans="1:10" hidden="1">
       <c r="A75" t="s">
         <v>6</v>
       </c>
@@ -10499,20 +10491,20 @@
       <c r="F75" t="s">
         <v>102</v>
       </c>
-      <c r="G75" s="108">
+      <c r="G75" s="102">
         <v>0</v>
       </c>
       <c r="H75" s="89">
         <v>0</v>
       </c>
-      <c r="I75" s="108">
+      <c r="I75" s="102">
         <v>0</v>
       </c>
-      <c r="J75" s="109">
+      <c r="J75" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:10">
+    <row r="76" spans="1:10" hidden="1">
       <c r="A76" t="s">
         <v>6</v>
       </c>
@@ -10531,20 +10523,20 @@
       <c r="F76" t="s">
         <v>105</v>
       </c>
-      <c r="G76" s="108">
+      <c r="G76" s="102">
         <v>0</v>
       </c>
       <c r="H76" s="89">
         <v>0</v>
       </c>
-      <c r="I76" s="108">
+      <c r="I76" s="102">
         <v>12</v>
       </c>
-      <c r="J76" s="109">
+      <c r="J76" s="107">
         <v>18</v>
       </c>
     </row>
-    <row r="77" spans="1:10">
+    <row r="77" spans="1:10" hidden="1">
       <c r="A77" t="s">
         <v>6</v>
       </c>
@@ -10563,20 +10555,20 @@
       <c r="F77" t="s">
         <v>108</v>
       </c>
-      <c r="G77" s="108">
+      <c r="G77" s="102">
         <v>2</v>
       </c>
       <c r="H77" s="89">
         <v>0</v>
       </c>
-      <c r="I77" s="108">
+      <c r="I77" s="102">
         <v>10</v>
       </c>
-      <c r="J77" s="109">
+      <c r="J77" s="107">
         <v>13</v>
       </c>
     </row>
-    <row r="78" spans="1:10">
+    <row r="78" spans="1:10" hidden="1">
       <c r="A78" t="s">
         <v>6</v>
       </c>
@@ -10595,20 +10587,20 @@
       <c r="F78" t="s">
         <v>111</v>
       </c>
-      <c r="G78" s="108">
+      <c r="G78" s="102">
         <v>0</v>
       </c>
       <c r="H78" s="89">
         <v>0</v>
       </c>
-      <c r="I78" s="108">
+      <c r="I78" s="102">
         <v>0</v>
       </c>
-      <c r="J78" s="109">
+      <c r="J78" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:10">
+    <row r="79" spans="1:10" hidden="1">
       <c r="A79" t="s">
         <v>6</v>
       </c>
@@ -10627,20 +10619,20 @@
       <c r="F79" t="s">
         <v>114</v>
       </c>
-      <c r="G79" s="108">
+      <c r="G79" s="102">
         <v>0</v>
       </c>
       <c r="H79" s="89">
         <v>0</v>
       </c>
-      <c r="I79" s="108">
+      <c r="I79" s="102">
         <v>10</v>
       </c>
-      <c r="J79" s="109">
+      <c r="J79" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:10">
+    <row r="80" spans="1:10" hidden="1">
       <c r="A80" s="88" t="s">
         <v>6</v>
       </c>
@@ -10659,20 +10651,20 @@
       <c r="F80" s="88" t="s">
         <v>117</v>
       </c>
-      <c r="G80" s="112">
+      <c r="G80" s="110">
         <v>0</v>
       </c>
-      <c r="H80" s="116">
+      <c r="H80" s="114">
         <v>0</v>
       </c>
-      <c r="I80" s="112">
+      <c r="I80" s="110">
         <v>0</v>
       </c>
-      <c r="J80" s="113">
+      <c r="J80" s="111">
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:10">
+    <row r="81" spans="1:10" hidden="1">
       <c r="A81" t="s">
         <v>6</v>
       </c>
@@ -10691,20 +10683,20 @@
       <c r="F81" t="s">
         <v>122</v>
       </c>
-      <c r="G81" s="108">
+      <c r="G81" s="102">
         <v>0</v>
       </c>
       <c r="H81" s="89">
         <v>0</v>
       </c>
-      <c r="I81" s="108">
+      <c r="I81" s="102">
         <v>0</v>
       </c>
-      <c r="J81" s="109">
+      <c r="J81" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:10">
+    <row r="82" spans="1:10" hidden="1">
       <c r="A82" t="s">
         <v>6</v>
       </c>
@@ -10723,20 +10715,20 @@
       <c r="F82" t="s">
         <v>167</v>
       </c>
-      <c r="G82" s="108">
+      <c r="G82" s="102">
         <v>0</v>
       </c>
       <c r="H82" s="89">
         <v>0</v>
       </c>
-      <c r="I82" s="108">
+      <c r="I82" s="102">
         <v>0</v>
       </c>
-      <c r="J82" s="109">
+      <c r="J82" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:10">
+    <row r="83" spans="1:10" hidden="1">
       <c r="A83" t="s">
         <v>6</v>
       </c>
@@ -10755,20 +10747,20 @@
       <c r="F83" t="s">
         <v>139</v>
       </c>
-      <c r="G83" s="108">
+      <c r="G83" s="102">
         <v>0</v>
       </c>
       <c r="H83" s="89">
         <v>0</v>
       </c>
-      <c r="I83" s="108">
+      <c r="I83" s="102">
         <v>0</v>
       </c>
-      <c r="J83" s="109">
+      <c r="J83" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:10">
+    <row r="84" spans="1:10" hidden="1">
       <c r="A84" t="s">
         <v>6</v>
       </c>
@@ -10787,20 +10779,20 @@
       <c r="F84" t="s">
         <v>142</v>
       </c>
-      <c r="G84" s="108">
+      <c r="G84" s="102">
         <v>2</v>
       </c>
       <c r="H84" s="89">
         <v>0</v>
       </c>
-      <c r="I84" s="108">
+      <c r="I84" s="102">
         <v>10</v>
       </c>
-      <c r="J84" s="109">
+      <c r="J84" s="107">
         <v>13</v>
       </c>
     </row>
-    <row r="85" spans="1:10">
+    <row r="85" spans="1:10" hidden="1">
       <c r="A85" t="s">
         <v>6</v>
       </c>
@@ -10819,20 +10811,20 @@
       <c r="F85" t="s">
         <v>139</v>
       </c>
-      <c r="G85" s="108">
+      <c r="G85" s="102">
         <v>0</v>
       </c>
       <c r="H85" s="89">
         <v>0</v>
       </c>
-      <c r="I85" s="108">
+      <c r="I85" s="102">
         <v>0</v>
       </c>
-      <c r="J85" s="109">
+      <c r="J85" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:10">
+    <row r="86" spans="1:10" hidden="1">
       <c r="A86" t="s">
         <v>6</v>
       </c>
@@ -10851,20 +10843,20 @@
       <c r="F86" t="s">
         <v>122</v>
       </c>
-      <c r="G86" s="108">
+      <c r="G86" s="102">
         <v>0</v>
       </c>
       <c r="H86" s="89">
         <v>0</v>
       </c>
-      <c r="I86" s="108">
+      <c r="I86" s="102">
         <v>0</v>
       </c>
-      <c r="J86" s="109">
+      <c r="J86" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:10">
+    <row r="87" spans="1:10" hidden="1">
       <c r="A87" t="s">
         <v>6</v>
       </c>
@@ -10883,20 +10875,20 @@
       <c r="F87" t="s">
         <v>142</v>
       </c>
-      <c r="G87" s="108">
+      <c r="G87" s="102">
         <v>0</v>
       </c>
       <c r="H87" s="89">
         <v>0</v>
       </c>
-      <c r="I87" s="108">
+      <c r="I87" s="102">
         <v>0</v>
       </c>
-      <c r="J87" s="109">
+      <c r="J87" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:10">
+    <row r="88" spans="1:10" hidden="1">
       <c r="A88" t="s">
         <v>6</v>
       </c>
@@ -10915,20 +10907,20 @@
       <c r="F88" t="s">
         <v>122</v>
       </c>
-      <c r="G88" s="108">
+      <c r="G88" s="102">
         <v>0</v>
       </c>
       <c r="H88" s="89">
         <v>0</v>
       </c>
-      <c r="I88" s="108">
+      <c r="I88" s="102">
         <v>0</v>
       </c>
-      <c r="J88" s="109">
+      <c r="J88" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:10">
+    <row r="89" spans="1:10" hidden="1">
       <c r="A89" t="s">
         <v>6</v>
       </c>
@@ -10947,20 +10939,20 @@
       <c r="F89" t="s">
         <v>124</v>
       </c>
-      <c r="G89" s="108">
+      <c r="G89" s="102">
         <v>0</v>
       </c>
       <c r="H89" s="89">
         <v>0</v>
       </c>
-      <c r="I89" s="108">
+      <c r="I89" s="102">
         <v>0</v>
       </c>
-      <c r="J89" s="109">
+      <c r="J89" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:10">
+    <row r="90" spans="1:10" hidden="1">
       <c r="A90" t="s">
         <v>6</v>
       </c>
@@ -10979,20 +10971,20 @@
       <c r="F90" t="s">
         <v>154</v>
       </c>
-      <c r="G90" s="108">
+      <c r="G90" s="102">
         <v>0</v>
       </c>
       <c r="H90" s="89">
         <v>0</v>
       </c>
-      <c r="I90" s="108">
+      <c r="I90" s="102">
         <v>0</v>
       </c>
-      <c r="J90" s="109">
+      <c r="J90" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:10">
+    <row r="91" spans="1:10" hidden="1">
       <c r="A91" t="s">
         <v>6</v>
       </c>
@@ -11011,20 +11003,20 @@
       <c r="F91" t="s">
         <v>157</v>
       </c>
-      <c r="G91" s="108">
+      <c r="G91" s="102">
         <v>0</v>
       </c>
       <c r="H91" s="89">
         <v>0</v>
       </c>
-      <c r="I91" s="108">
+      <c r="I91" s="102">
         <v>0</v>
       </c>
-      <c r="J91" s="109">
+      <c r="J91" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:10">
+    <row r="92" spans="1:10" hidden="1">
       <c r="A92" t="s">
         <v>6</v>
       </c>
@@ -11043,20 +11035,20 @@
       <c r="F92" t="s">
         <v>128</v>
       </c>
-      <c r="G92" s="108">
+      <c r="G92" s="102">
         <v>0</v>
       </c>
       <c r="H92" s="89">
         <v>0</v>
       </c>
-      <c r="I92" s="108">
+      <c r="I92" s="102">
         <v>0</v>
       </c>
-      <c r="J92" s="109">
+      <c r="J92" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:10">
+    <row r="93" spans="1:10" hidden="1">
       <c r="A93" t="s">
         <v>6</v>
       </c>
@@ -11075,20 +11067,20 @@
       <c r="F93" t="s">
         <v>145</v>
       </c>
-      <c r="G93" s="108">
+      <c r="G93" s="102">
         <v>0</v>
       </c>
       <c r="H93" s="89">
         <v>0</v>
       </c>
-      <c r="I93" s="108">
+      <c r="I93" s="102">
         <v>0</v>
       </c>
-      <c r="J93" s="109">
+      <c r="J93" s="107">
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:10">
+    <row r="94" spans="1:10" hidden="1">
       <c r="A94" s="88" t="s">
         <v>6</v>
       </c>
@@ -11107,16 +11099,16 @@
       <c r="F94" s="88" t="s">
         <v>159</v>
       </c>
-      <c r="G94" s="112">
+      <c r="G94" s="110">
         <v>0</v>
       </c>
-      <c r="H94" s="116">
+      <c r="H94" s="114">
         <v>0</v>
       </c>
-      <c r="I94" s="112">
+      <c r="I94" s="110">
         <v>0</v>
       </c>
-      <c r="J94" s="112">
+      <c r="J94" s="110">
         <v>0</v>
       </c>
     </row>
@@ -11127,7 +11119,7 @@
       <c r="B95" t="s">
         <v>1</v>
       </c>
-      <c r="C95" s="114" t="s">
+      <c r="C95" s="112" t="s">
         <v>19</v>
       </c>
       <c r="D95" t="s">
@@ -11136,19 +11128,19 @@
       <c r="E95" t="s">
         <v>176</v>
       </c>
-      <c r="F95" s="114" t="s">
+      <c r="F95" s="112" t="s">
         <v>745</v>
       </c>
-      <c r="G95" s="115">
+      <c r="G95" s="113">
         <v>0</v>
       </c>
-      <c r="H95" s="102">
+      <c r="H95" s="89">
         <v>0</v>
       </c>
-      <c r="I95" s="103">
+      <c r="I95" s="102">
         <v>0</v>
       </c>
-      <c r="J95" s="103">
+      <c r="J95" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11159,7 +11151,7 @@
       <c r="B96" t="s">
         <v>1</v>
       </c>
-      <c r="C96" s="114" t="s">
+      <c r="C96" s="112" t="s">
         <v>19</v>
       </c>
       <c r="D96" t="s">
@@ -11168,19 +11160,19 @@
       <c r="E96" t="s">
         <v>178</v>
       </c>
-      <c r="F96" s="114" t="s">
+      <c r="F96" s="112" t="s">
         <v>746</v>
       </c>
-      <c r="G96" s="115">
+      <c r="G96" s="113">
         <v>0</v>
       </c>
-      <c r="H96" s="102">
+      <c r="H96" s="89">
         <v>0</v>
       </c>
-      <c r="I96" s="103">
+      <c r="I96" s="102">
         <v>0</v>
       </c>
-      <c r="J96" s="103">
+      <c r="J96" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11191,7 +11183,7 @@
       <c r="B97" t="s">
         <v>1</v>
       </c>
-      <c r="C97" s="114" t="s">
+      <c r="C97" s="112" t="s">
         <v>19</v>
       </c>
       <c r="D97" t="s">
@@ -11200,19 +11192,19 @@
       <c r="E97" t="s">
         <v>180</v>
       </c>
-      <c r="F97" s="114" t="s">
+      <c r="F97" s="112" t="s">
         <v>747</v>
       </c>
-      <c r="G97" s="115">
+      <c r="G97" s="113">
         <v>0</v>
       </c>
-      <c r="H97" s="102">
+      <c r="H97" s="89">
         <v>0</v>
       </c>
-      <c r="I97" s="103">
+      <c r="I97" s="102">
         <v>0</v>
       </c>
-      <c r="J97" s="103">
+      <c r="J97" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11223,7 +11215,7 @@
       <c r="B98" t="s">
         <v>1</v>
       </c>
-      <c r="C98" s="114" t="s">
+      <c r="C98" s="112" t="s">
         <v>19</v>
       </c>
       <c r="D98" t="s">
@@ -11232,19 +11224,19 @@
       <c r="E98" t="s">
         <v>182</v>
       </c>
-      <c r="F98" s="114" t="s">
+      <c r="F98" s="112" t="s">
         <v>748</v>
       </c>
-      <c r="G98" s="115">
+      <c r="G98" s="113">
         <v>0</v>
       </c>
-      <c r="H98" s="102">
+      <c r="H98" s="89">
         <v>0</v>
       </c>
-      <c r="I98" s="103">
+      <c r="I98" s="102">
         <v>0</v>
       </c>
-      <c r="J98" s="103">
+      <c r="J98" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11255,7 +11247,7 @@
       <c r="B99" t="s">
         <v>1</v>
       </c>
-      <c r="C99" s="114" t="s">
+      <c r="C99" s="112" t="s">
         <v>19</v>
       </c>
       <c r="D99" t="s">
@@ -11264,30 +11256,30 @@
       <c r="E99" t="s">
         <v>184</v>
       </c>
-      <c r="F99" s="114" t="s">
+      <c r="F99" s="112" t="s">
         <v>749</v>
       </c>
-      <c r="G99" s="115">
+      <c r="G99" s="113">
         <v>0</v>
       </c>
-      <c r="H99" s="102">
+      <c r="H99" s="89">
         <v>0</v>
       </c>
-      <c r="I99" s="103">
+      <c r="I99" s="102">
         <v>0</v>
       </c>
-      <c r="J99" s="103">
+      <c r="J99" s="102">
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:10">
+    <row r="100" spans="1:10" hidden="1">
       <c r="A100" s="88" t="s">
         <v>6</v>
       </c>
       <c r="B100" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="C100" s="119" t="s">
+      <c r="C100" s="117" t="s">
         <v>19</v>
       </c>
       <c r="D100" s="88" t="s">
@@ -11296,51 +11288,51 @@
       <c r="E100" s="88" t="s">
         <v>186</v>
       </c>
-      <c r="F100" s="119" t="s">
+      <c r="F100" s="117" t="s">
         <v>750</v>
       </c>
-      <c r="G100" s="117">
+      <c r="G100" s="115">
         <v>0</v>
       </c>
-      <c r="H100" s="116">
+      <c r="H100" s="114">
         <v>0</v>
       </c>
-      <c r="I100" s="112">
+      <c r="I100" s="110">
         <v>0</v>
       </c>
-      <c r="J100" s="112">
+      <c r="J100" s="110">
         <v>0</v>
       </c>
     </row>
     <row r="101" spans="1:10">
-      <c r="A101" s="120" t="s">
+      <c r="A101" t="s">
         <v>7</v>
       </c>
-      <c r="B101" s="120" t="s">
+      <c r="B101" t="s">
         <v>1</v>
       </c>
-      <c r="C101" s="121" t="s">
+      <c r="C101" s="112" t="s">
         <v>758</v>
       </c>
-      <c r="D101" s="120" t="s">
+      <c r="D101" t="s">
         <v>333</v>
       </c>
-      <c r="E101" s="120" t="s">
+      <c r="E101" t="s">
         <v>92</v>
       </c>
-      <c r="F101" s="121" t="s">
+      <c r="F101" s="112" t="s">
         <v>93</v>
       </c>
-      <c r="G101" s="122">
+      <c r="G101" s="113">
         <v>0</v>
       </c>
-      <c r="H101" s="102">
+      <c r="H101" s="89">
         <v>0</v>
       </c>
-      <c r="I101" s="103">
+      <c r="I101" s="102">
         <v>0</v>
       </c>
-      <c r="J101" s="103">
+      <c r="J101" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11351,7 +11343,7 @@
       <c r="B102" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="C102" s="119" t="s">
+      <c r="C102" s="117" t="s">
         <v>758</v>
       </c>
       <c r="D102" s="88" t="s">
@@ -11360,19 +11352,19 @@
       <c r="E102" s="88" t="s">
         <v>110</v>
       </c>
-      <c r="F102" s="119" t="s">
+      <c r="F102" s="117" t="s">
         <v>111</v>
       </c>
-      <c r="G102" s="117">
+      <c r="G102" s="115">
         <v>0</v>
       </c>
-      <c r="H102" s="116">
+      <c r="H102" s="114">
         <v>0</v>
       </c>
-      <c r="I102" s="112">
+      <c r="I102" s="110">
         <v>0</v>
       </c>
-      <c r="J102" s="112">
+      <c r="J102" s="110">
         <v>0</v>
       </c>
     </row>
@@ -11383,7 +11375,7 @@
       <c r="B103" t="s">
         <v>1</v>
       </c>
-      <c r="C103" s="114" t="s">
+      <c r="C103" s="112" t="s">
         <v>118</v>
       </c>
       <c r="D103" t="s">
@@ -11392,19 +11384,19 @@
       <c r="E103" t="s">
         <v>188</v>
       </c>
-      <c r="F103" s="114" t="s">
+      <c r="F103" s="112" t="s">
         <v>751</v>
       </c>
-      <c r="G103" s="115">
+      <c r="G103" s="113">
         <v>0</v>
       </c>
-      <c r="H103" s="102">
+      <c r="H103" s="89">
         <v>0</v>
       </c>
-      <c r="I103" s="103">
+      <c r="I103" s="102">
         <v>0</v>
       </c>
-      <c r="J103" s="103">
+      <c r="J103" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11415,28 +11407,28 @@
       <c r="B104" t="s">
         <v>1</v>
       </c>
-      <c r="C104" s="114" t="s">
+      <c r="C104" s="112" t="s">
         <v>118</v>
       </c>
       <c r="D104" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E104" t="s">
-        <v>188</v>
-      </c>
-      <c r="F104" s="114" t="s">
-        <v>751</v>
-      </c>
-      <c r="G104" s="115">
+        <v>190</v>
+      </c>
+      <c r="F104" s="112" t="s">
+        <v>756</v>
+      </c>
+      <c r="G104" s="113">
         <v>0</v>
       </c>
-      <c r="H104" s="102">
+      <c r="H104" s="89">
         <v>0</v>
       </c>
-      <c r="I104" s="103">
+      <c r="I104" s="102">
         <v>0</v>
       </c>
-      <c r="J104" s="103">
+      <c r="J104" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11447,28 +11439,28 @@
       <c r="B105" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="C105" s="119" t="s">
-        <v>118</v>
+      <c r="C105" s="117" t="s">
+        <v>19</v>
       </c>
       <c r="D105" s="88" t="s">
-        <v>189</v>
+        <v>210</v>
       </c>
       <c r="E105" s="88" t="s">
-        <v>190</v>
-      </c>
-      <c r="F105" s="119" t="s">
-        <v>756</v>
-      </c>
-      <c r="G105" s="117">
+        <v>186</v>
+      </c>
+      <c r="F105" s="117" t="s">
+        <v>750</v>
+      </c>
+      <c r="G105" s="115">
         <v>0</v>
       </c>
-      <c r="H105" s="116">
+      <c r="H105" s="114">
         <v>0</v>
       </c>
-      <c r="I105" s="112">
+      <c r="I105" s="110">
         <v>0</v>
       </c>
-      <c r="J105" s="112">
+      <c r="J105" s="110">
         <v>0</v>
       </c>
     </row>
@@ -11479,7 +11471,7 @@
       <c r="B106" t="s">
         <v>1</v>
       </c>
-      <c r="C106" s="114" t="s">
+      <c r="C106" s="112" t="s">
         <v>132</v>
       </c>
       <c r="D106" t="s">
@@ -11488,19 +11480,19 @@
       <c r="E106" t="s">
         <v>192</v>
       </c>
-      <c r="F106" s="114" t="s">
+      <c r="F106" s="112" t="s">
         <v>752</v>
       </c>
-      <c r="G106" s="115">
+      <c r="G106" s="113">
         <v>0</v>
       </c>
-      <c r="H106" s="102">
+      <c r="H106" s="89">
         <v>0</v>
       </c>
-      <c r="I106" s="103">
+      <c r="I106" s="102">
         <v>0</v>
       </c>
-      <c r="J106" s="103">
+      <c r="J106" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11511,7 +11503,7 @@
       <c r="B107" t="s">
         <v>1</v>
       </c>
-      <c r="C107" s="114" t="s">
+      <c r="C107" s="112" t="s">
         <v>132</v>
       </c>
       <c r="D107" t="s">
@@ -11520,19 +11512,19 @@
       <c r="E107" t="s">
         <v>192</v>
       </c>
-      <c r="F107" s="114" t="s">
+      <c r="F107" s="112" t="s">
         <v>752</v>
       </c>
-      <c r="G107" s="115">
+      <c r="G107" s="113">
         <v>0</v>
       </c>
-      <c r="H107" s="102">
+      <c r="H107" s="89">
         <v>0</v>
       </c>
-      <c r="I107" s="103">
+      <c r="I107" s="102">
         <v>0</v>
       </c>
-      <c r="J107" s="103">
+      <c r="J107" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11543,7 +11535,7 @@
       <c r="B108" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="C108" s="119" t="s">
+      <c r="C108" s="117" t="s">
         <v>132</v>
       </c>
       <c r="D108" s="88" t="s">
@@ -11552,19 +11544,19 @@
       <c r="E108" s="88" t="s">
         <v>334</v>
       </c>
-      <c r="F108" s="119" t="s">
+      <c r="F108" s="117" t="s">
         <v>757</v>
       </c>
-      <c r="G108" s="117">
+      <c r="G108" s="115">
         <v>0</v>
       </c>
-      <c r="H108" s="116">
+      <c r="H108" s="114">
         <v>0</v>
       </c>
-      <c r="I108" s="112">
+      <c r="I108" s="110">
         <v>0</v>
       </c>
-      <c r="J108" s="112">
+      <c r="J108" s="110">
         <v>0</v>
       </c>
     </row>
@@ -11575,7 +11567,7 @@
       <c r="B109" t="s">
         <v>1</v>
       </c>
-      <c r="C109" s="114" t="s">
+      <c r="C109" s="112" t="s">
         <v>148</v>
       </c>
       <c r="D109" t="s">
@@ -11584,19 +11576,19 @@
       <c r="E109" t="s">
         <v>195</v>
       </c>
-      <c r="F109" s="114" t="s">
+      <c r="F109" s="112" t="s">
         <v>753</v>
       </c>
-      <c r="G109" s="115">
+      <c r="G109" s="113">
         <v>0</v>
       </c>
-      <c r="H109" s="102">
+      <c r="H109" s="89">
         <v>0</v>
       </c>
-      <c r="I109" s="103">
+      <c r="I109" s="102">
         <v>0</v>
       </c>
-      <c r="J109" s="103">
+      <c r="J109" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11607,7 +11599,7 @@
       <c r="B110" t="s">
         <v>1</v>
       </c>
-      <c r="C110" s="114" t="s">
+      <c r="C110" s="112" t="s">
         <v>148</v>
       </c>
       <c r="D110" t="s">
@@ -11616,19 +11608,19 @@
       <c r="E110" t="s">
         <v>335</v>
       </c>
-      <c r="F110" s="114" t="s">
+      <c r="F110" s="112" t="s">
         <v>754</v>
       </c>
-      <c r="G110" s="115">
+      <c r="G110" s="113">
         <v>0</v>
       </c>
-      <c r="H110" s="102">
+      <c r="H110" s="89">
         <v>0</v>
       </c>
-      <c r="I110" s="103">
+      <c r="I110" s="102">
         <v>0</v>
       </c>
-      <c r="J110" s="103">
+      <c r="J110" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11639,7 +11631,7 @@
       <c r="B111" t="s">
         <v>1</v>
       </c>
-      <c r="C111" s="114" t="s">
+      <c r="C111" s="112" t="s">
         <v>148</v>
       </c>
       <c r="D111" t="s">
@@ -11648,19 +11640,19 @@
       <c r="E111" t="s">
         <v>197</v>
       </c>
-      <c r="F111" s="114" t="s">
+      <c r="F111" s="112" t="s">
         <v>755</v>
       </c>
-      <c r="G111" s="115">
+      <c r="G111" s="113">
         <v>0</v>
       </c>
-      <c r="H111" s="102">
+      <c r="H111" s="89">
         <v>0</v>
       </c>
-      <c r="I111" s="103">
+      <c r="I111" s="102">
         <v>0</v>
       </c>
-      <c r="J111" s="103">
+      <c r="J111" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11671,7 +11663,7 @@
       <c r="B112" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="C112" s="119" t="s">
+      <c r="C112" s="117" t="s">
         <v>148</v>
       </c>
       <c r="D112" s="88" t="s">
@@ -11680,19 +11672,19 @@
       <c r="E112" s="88" t="s">
         <v>336</v>
       </c>
-      <c r="F112" s="119" t="s">
+      <c r="F112" s="117" t="s">
         <v>759</v>
       </c>
-      <c r="G112" s="117">
+      <c r="G112" s="115">
         <v>0</v>
       </c>
-      <c r="H112" s="116">
+      <c r="H112" s="114">
         <v>0</v>
       </c>
-      <c r="I112" s="112">
+      <c r="I112" s="110">
         <v>0</v>
       </c>
-      <c r="J112" s="112">
+      <c r="J112" s="110">
         <v>0</v>
       </c>
     </row>
@@ -11703,7 +11695,7 @@
       <c r="B113" t="s">
         <v>1</v>
       </c>
-      <c r="C113" s="114" t="s">
+      <c r="C113" s="112" t="s">
         <v>760</v>
       </c>
       <c r="D113" t="s">
@@ -11712,22 +11704,22 @@
       <c r="E113" t="s">
         <v>92</v>
       </c>
-      <c r="F113" s="114" t="s">
+      <c r="F113" s="112" t="s">
         <v>93</v>
       </c>
-      <c r="G113" s="115">
+      <c r="G113" s="113">
         <v>0</v>
       </c>
-      <c r="H113" s="102">
+      <c r="H113" s="89">
         <v>0</v>
       </c>
-      <c r="I113" s="103">
+      <c r="I113" s="102">
         <v>0</v>
       </c>
-      <c r="J113" s="103">
+      <c r="J113" s="102">
         <v>0</v>
       </c>
-      <c r="K113" s="118" t="s">
+      <c r="K113" s="116" t="s">
         <v>743</v>
       </c>
     </row>
@@ -11747,19 +11739,19 @@
       <c r="E114" t="s">
         <v>110</v>
       </c>
-      <c r="F114" s="114" t="s">
+      <c r="F114" s="112" t="s">
         <v>111</v>
       </c>
-      <c r="G114" s="115">
+      <c r="G114" s="113">
         <v>0</v>
       </c>
-      <c r="H114" s="102">
+      <c r="H114" s="89">
         <v>0</v>
       </c>
-      <c r="I114" s="103">
+      <c r="I114" s="102">
         <v>0</v>
       </c>
-      <c r="J114" s="103">
+      <c r="J114" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11779,19 +11771,19 @@
       <c r="E115" t="s">
         <v>188</v>
       </c>
-      <c r="F115" s="114" t="s">
+      <c r="F115" s="112" t="s">
         <v>751</v>
       </c>
-      <c r="G115" s="115">
+      <c r="G115" s="113">
         <v>0</v>
       </c>
-      <c r="H115" s="102">
+      <c r="H115" s="89">
         <v>0</v>
       </c>
-      <c r="I115" s="103">
+      <c r="I115" s="102">
         <v>0</v>
       </c>
-      <c r="J115" s="103">
+      <c r="J115" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11811,19 +11803,19 @@
       <c r="E116" t="s">
         <v>188</v>
       </c>
-      <c r="F116" s="114" t="s">
+      <c r="F116" s="112" t="s">
         <v>751</v>
       </c>
-      <c r="G116" s="115">
+      <c r="G116" s="113">
         <v>0</v>
       </c>
-      <c r="H116" s="102">
+      <c r="H116" s="89">
         <v>0</v>
       </c>
-      <c r="I116" s="103">
+      <c r="I116" s="102">
         <v>0</v>
       </c>
-      <c r="J116" s="103">
+      <c r="J116" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11843,19 +11835,19 @@
       <c r="E117" t="s">
         <v>101</v>
       </c>
-      <c r="F117" s="114" t="s">
+      <c r="F117" s="112" t="s">
         <v>102</v>
       </c>
-      <c r="G117" s="115">
+      <c r="G117" s="113">
         <v>0</v>
       </c>
-      <c r="H117" s="102">
+      <c r="H117" s="89">
         <v>0</v>
       </c>
-      <c r="I117" s="103">
+      <c r="I117" s="102">
         <v>0</v>
       </c>
-      <c r="J117" s="103">
+      <c r="J117" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11875,19 +11867,19 @@
       <c r="E118" t="s">
         <v>101</v>
       </c>
-      <c r="F118" s="114" t="s">
+      <c r="F118" s="112" t="s">
         <v>102</v>
       </c>
-      <c r="G118" s="115">
+      <c r="G118" s="113">
         <v>0</v>
       </c>
-      <c r="H118" s="102">
+      <c r="H118" s="89">
         <v>0</v>
       </c>
-      <c r="I118" s="103">
+      <c r="I118" s="102">
         <v>0</v>
       </c>
-      <c r="J118" s="103">
+      <c r="J118" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11907,19 +11899,19 @@
       <c r="E119" t="s">
         <v>107</v>
       </c>
-      <c r="F119" s="114" t="s">
+      <c r="F119" s="112" t="s">
         <v>108</v>
       </c>
-      <c r="G119" s="115">
+      <c r="G119" s="113">
         <v>0</v>
       </c>
-      <c r="H119" s="102">
+      <c r="H119" s="89">
         <v>0</v>
       </c>
-      <c r="I119" s="103">
+      <c r="I119" s="102">
         <v>0</v>
       </c>
-      <c r="J119" s="103">
+      <c r="J119" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11939,19 +11931,19 @@
       <c r="E120" t="s">
         <v>101</v>
       </c>
-      <c r="F120" s="114" t="s">
+      <c r="F120" s="112" t="s">
         <v>102</v>
       </c>
-      <c r="G120" s="115">
+      <c r="G120" s="113">
         <v>0</v>
       </c>
-      <c r="H120" s="102">
+      <c r="H120" s="89">
         <v>0</v>
       </c>
-      <c r="I120" s="103">
+      <c r="I120" s="102">
         <v>0</v>
       </c>
-      <c r="J120" s="103">
+      <c r="J120" s="102">
         <v>0</v>
       </c>
     </row>
@@ -11971,19 +11963,19 @@
       <c r="E121" s="88" t="s">
         <v>116</v>
       </c>
-      <c r="F121" s="119" t="s">
+      <c r="F121" s="117" t="s">
         <v>87</v>
       </c>
-      <c r="G121" s="117">
+      <c r="G121" s="115">
         <v>0</v>
       </c>
-      <c r="H121" s="116">
+      <c r="H121" s="114">
         <v>0</v>
       </c>
-      <c r="I121" s="112">
+      <c r="I121" s="110">
         <v>0</v>
       </c>
-      <c r="J121" s="112">
+      <c r="J121" s="110">
         <v>0</v>
       </c>
     </row>
@@ -11994,7 +11986,7 @@
       <c r="B122" t="s">
         <v>2</v>
       </c>
-      <c r="C122" s="114" t="s">
+      <c r="C122" s="112" t="s">
         <v>19</v>
       </c>
       <c r="D122" t="s">
@@ -12003,19 +11995,19 @@
       <c r="E122" t="s">
         <v>176</v>
       </c>
-      <c r="F122" s="114" t="s">
+      <c r="F122" s="112" t="s">
         <v>745</v>
       </c>
-      <c r="G122" s="115">
+      <c r="G122" s="113">
         <v>0</v>
       </c>
-      <c r="H122" s="102">
+      <c r="H122" s="89">
         <v>0</v>
       </c>
-      <c r="I122" s="103">
+      <c r="I122" s="102">
         <v>0</v>
       </c>
-      <c r="J122" s="103">
+      <c r="J122" s="102">
         <v>0</v>
       </c>
       <c r="K122" t="s">
@@ -12038,19 +12030,19 @@
       <c r="E123" t="s">
         <v>178</v>
       </c>
-      <c r="F123" s="114" t="s">
+      <c r="F123" s="112" t="s">
         <v>746</v>
       </c>
-      <c r="G123" s="115">
+      <c r="G123" s="113">
         <v>0</v>
       </c>
-      <c r="H123" s="102">
+      <c r="H123" s="89">
         <v>0</v>
       </c>
-      <c r="I123" s="103">
+      <c r="I123" s="102">
         <v>0</v>
       </c>
-      <c r="J123" s="103">
+      <c r="J123" s="102">
         <v>0</v>
       </c>
     </row>
@@ -12070,19 +12062,19 @@
       <c r="E124" t="s">
         <v>182</v>
       </c>
-      <c r="F124" s="114" t="s">
+      <c r="F124" s="112" t="s">
         <v>748</v>
       </c>
-      <c r="G124" s="115">
+      <c r="G124" s="113">
         <v>0</v>
       </c>
-      <c r="H124" s="102">
+      <c r="H124" s="89">
         <v>0</v>
       </c>
-      <c r="I124" s="103">
+      <c r="I124" s="102">
         <v>0</v>
       </c>
-      <c r="J124" s="103">
+      <c r="J124" s="102">
         <v>0</v>
       </c>
     </row>
@@ -12102,19 +12094,19 @@
       <c r="E125" t="s">
         <v>184</v>
       </c>
-      <c r="F125" s="114" t="s">
+      <c r="F125" s="112" t="s">
         <v>749</v>
       </c>
-      <c r="G125" s="115">
+      <c r="G125" s="113">
         <v>0</v>
       </c>
-      <c r="H125" s="102">
+      <c r="H125" s="89">
         <v>0</v>
       </c>
-      <c r="I125" s="103">
+      <c r="I125" s="102">
         <v>0</v>
       </c>
-      <c r="J125" s="103">
+      <c r="J125" s="102">
         <v>0</v>
       </c>
     </row>
@@ -12134,19 +12126,19 @@
       <c r="E126" s="88" t="s">
         <v>186</v>
       </c>
-      <c r="F126" s="119" t="s">
+      <c r="F126" s="117" t="s">
         <v>750</v>
       </c>
-      <c r="G126" s="117">
+      <c r="G126" s="115">
         <v>0</v>
       </c>
-      <c r="H126" s="116">
+      <c r="H126" s="114">
         <v>0</v>
       </c>
-      <c r="I126" s="112">
+      <c r="I126" s="110">
         <v>0</v>
       </c>
-      <c r="J126" s="112">
+      <c r="J126" s="110">
         <v>0</v>
       </c>
     </row>
@@ -12157,7 +12149,7 @@
       <c r="B127" t="s">
         <v>2</v>
       </c>
-      <c r="C127" s="114" t="s">
+      <c r="C127" s="112" t="s">
         <v>118</v>
       </c>
       <c r="D127" t="s">
@@ -12166,19 +12158,19 @@
       <c r="E127" t="s">
         <v>188</v>
       </c>
-      <c r="F127" s="114" t="s">
+      <c r="F127" s="112" t="s">
         <v>751</v>
       </c>
-      <c r="G127" s="115">
+      <c r="G127" s="113">
         <v>0</v>
       </c>
-      <c r="H127" s="102">
+      <c r="H127" s="89">
         <v>0</v>
       </c>
-      <c r="I127" s="103">
+      <c r="I127" s="102">
         <v>0</v>
       </c>
-      <c r="J127" s="103">
+      <c r="J127" s="102">
         <v>0</v>
       </c>
     </row>
@@ -12189,7 +12181,7 @@
       <c r="B128" t="s">
         <v>2</v>
       </c>
-      <c r="C128" s="114" t="s">
+      <c r="C128" s="112" t="s">
         <v>118</v>
       </c>
       <c r="D128" t="s">
@@ -12198,51 +12190,51 @@
       <c r="E128" t="s">
         <v>188</v>
       </c>
-      <c r="F128" s="114" t="s">
+      <c r="F128" s="112" t="s">
         <v>751</v>
       </c>
-      <c r="G128" s="115">
+      <c r="G128" s="113">
         <v>0</v>
       </c>
-      <c r="H128" s="102">
+      <c r="H128" s="89">
         <v>0</v>
       </c>
-      <c r="I128" s="103">
+      <c r="I128" s="102">
         <v>0</v>
       </c>
-      <c r="J128" s="103">
+      <c r="J128" s="102">
         <v>0</v>
       </c>
     </row>
     <row r="129" spans="1:10">
-      <c r="A129" s="120" t="s">
+      <c r="A129" t="s">
         <v>7</v>
       </c>
-      <c r="B129" s="120" t="s">
+      <c r="B129" t="s">
         <v>2</v>
       </c>
-      <c r="C129" s="114" t="s">
+      <c r="C129" s="112" t="s">
         <v>118</v>
       </c>
-      <c r="D129" s="120" t="s">
+      <c r="D129" t="s">
         <v>213</v>
       </c>
-      <c r="E129" s="120" t="s">
+      <c r="E129" t="s">
         <v>188</v>
       </c>
-      <c r="F129" s="121" t="s">
+      <c r="F129" s="112" t="s">
         <v>751</v>
       </c>
-      <c r="G129" s="122">
+      <c r="G129" s="113">
         <v>0</v>
       </c>
-      <c r="H129" s="102">
+      <c r="H129" s="89">
         <v>0</v>
       </c>
-      <c r="I129" s="103">
+      <c r="I129" s="102">
         <v>0</v>
       </c>
-      <c r="J129" s="103">
+      <c r="J129" s="102">
         <v>0</v>
       </c>
     </row>
@@ -12253,7 +12245,7 @@
       <c r="B130" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="C130" s="119" t="s">
+      <c r="C130" s="117" t="s">
         <v>118</v>
       </c>
       <c r="D130" s="88" t="s">
@@ -12262,115 +12254,115 @@
       <c r="E130" s="88" t="s">
         <v>190</v>
       </c>
-      <c r="F130" s="119" t="s">
+      <c r="F130" s="117" t="s">
         <v>756</v>
       </c>
-      <c r="G130" s="117">
+      <c r="G130" s="115">
         <v>0</v>
       </c>
-      <c r="H130" s="116">
+      <c r="H130" s="114">
         <v>0</v>
       </c>
-      <c r="I130" s="112">
+      <c r="I130" s="110">
         <v>0</v>
       </c>
-      <c r="J130" s="112">
+      <c r="J130" s="110">
         <v>0</v>
       </c>
     </row>
     <row r="131" spans="1:10">
-      <c r="A131" s="120" t="s">
+      <c r="A131" t="s">
         <v>7</v>
       </c>
-      <c r="B131" s="120" t="s">
+      <c r="B131" t="s">
         <v>2</v>
       </c>
-      <c r="C131" s="121" t="s">
+      <c r="C131" s="112" t="s">
         <v>148</v>
       </c>
-      <c r="D131" s="120" t="s">
+      <c r="D131" t="s">
         <v>214</v>
       </c>
-      <c r="E131" s="120" t="s">
+      <c r="E131" t="s">
         <v>197</v>
       </c>
-      <c r="F131" s="121" t="s">
+      <c r="F131" s="112" t="s">
         <v>755</v>
       </c>
-      <c r="G131" s="122">
+      <c r="G131" s="113">
         <v>0</v>
       </c>
-      <c r="H131" s="102">
+      <c r="H131" s="89">
         <v>0</v>
       </c>
-      <c r="I131" s="103">
+      <c r="I131" s="102">
         <v>0</v>
       </c>
-      <c r="J131" s="103">
+      <c r="J131" s="102">
         <v>0</v>
       </c>
     </row>
     <row r="132" spans="1:10">
-      <c r="A132" s="120" t="s">
+      <c r="A132" t="s">
         <v>7</v>
       </c>
-      <c r="B132" s="120" t="s">
+      <c r="B132" t="s">
         <v>2</v>
       </c>
-      <c r="C132" s="121" t="s">
+      <c r="C132" s="112" t="s">
         <v>148</v>
       </c>
-      <c r="D132" s="120" t="s">
+      <c r="D132" t="s">
         <v>172</v>
       </c>
-      <c r="E132" s="120" t="s">
+      <c r="E132" t="s">
         <v>195</v>
       </c>
-      <c r="F132" s="121" t="s">
+      <c r="F132" s="112" t="s">
         <v>753</v>
       </c>
-      <c r="G132" s="122">
+      <c r="G132" s="113">
         <v>0</v>
       </c>
-      <c r="H132" s="102">
+      <c r="H132" s="89">
         <v>0</v>
       </c>
-      <c r="I132" s="103">
+      <c r="I132" s="102">
         <v>0</v>
       </c>
-      <c r="J132" s="103">
+      <c r="J132" s="102">
         <v>0</v>
       </c>
     </row>
     <row r="133" spans="1:10">
-      <c r="A133" s="120" t="s">
+      <c r="A133" t="s">
         <v>7</v>
       </c>
-      <c r="B133" s="120" t="s">
+      <c r="B133" t="s">
         <v>2</v>
       </c>
-      <c r="C133" s="121" t="s">
+      <c r="C133" s="112" t="s">
         <v>148</v>
       </c>
-      <c r="D133" s="120" t="s">
+      <c r="D133" t="s">
         <v>215</v>
       </c>
-      <c r="E133" s="120" t="s">
+      <c r="E133" t="s">
         <v>195</v>
       </c>
-      <c r="F133" s="121" t="s">
+      <c r="F133" s="112" t="s">
         <v>753</v>
       </c>
-      <c r="G133" s="122">
+      <c r="G133" s="113">
         <v>0</v>
       </c>
-      <c r="H133" s="102">
+      <c r="H133" s="89">
         <v>0</v>
       </c>
-      <c r="I133" s="103">
+      <c r="I133" s="102">
         <v>0</v>
       </c>
-      <c r="J133" s="103">
+      <c r="J133" s="102">
         <v>0</v>
       </c>
     </row>
@@ -12381,7 +12373,7 @@
       <c r="B134" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="C134" s="119" t="s">
+      <c r="C134" s="117" t="s">
         <v>148</v>
       </c>
       <c r="D134" s="88" t="s">
@@ -12390,147 +12382,147 @@
       <c r="E134" s="88" t="s">
         <v>336</v>
       </c>
-      <c r="F134" s="119" t="s">
+      <c r="F134" s="117" t="s">
         <v>759</v>
       </c>
-      <c r="G134" s="117">
+      <c r="G134" s="115">
         <v>0</v>
       </c>
-      <c r="H134" s="116">
+      <c r="H134" s="114">
         <v>0</v>
       </c>
-      <c r="I134" s="112">
+      <c r="I134" s="110">
         <v>0</v>
       </c>
-      <c r="J134" s="112">
+      <c r="J134" s="110">
         <v>0</v>
       </c>
     </row>
     <row r="135" spans="1:10">
-      <c r="A135" s="120" t="s">
+      <c r="A135" t="s">
         <v>7</v>
       </c>
-      <c r="B135" s="120" t="s">
+      <c r="B135" t="s">
         <v>2</v>
       </c>
-      <c r="C135" s="121" t="s">
+      <c r="C135" s="112" t="s">
         <v>132</v>
       </c>
-      <c r="D135" s="120" t="s">
+      <c r="D135" t="s">
         <v>216</v>
       </c>
-      <c r="E135" s="120" t="s">
+      <c r="E135" t="s">
         <v>192</v>
       </c>
-      <c r="F135" s="121" t="s">
+      <c r="F135" s="112" t="s">
         <v>752</v>
       </c>
-      <c r="G135" s="122">
+      <c r="G135" s="113">
         <v>0</v>
       </c>
-      <c r="H135" s="102">
+      <c r="H135" s="89">
         <v>0</v>
       </c>
-      <c r="I135" s="103">
+      <c r="I135" s="102">
         <v>0</v>
       </c>
-      <c r="J135" s="103">
+      <c r="J135" s="102">
         <v>0</v>
       </c>
     </row>
     <row r="136" spans="1:10">
-      <c r="A136" s="120" t="s">
+      <c r="A136" t="s">
         <v>7</v>
       </c>
-      <c r="B136" s="120" t="s">
+      <c r="B136" t="s">
         <v>2</v>
       </c>
-      <c r="C136" s="121" t="s">
+      <c r="C136" s="112" t="s">
         <v>132</v>
       </c>
-      <c r="D136" s="120" t="s">
+      <c r="D136" t="s">
         <v>217</v>
       </c>
-      <c r="E136" s="120" t="s">
+      <c r="E136" t="s">
         <v>192</v>
       </c>
-      <c r="F136" s="121" t="s">
+      <c r="F136" s="112" t="s">
         <v>752</v>
       </c>
-      <c r="G136" s="122">
+      <c r="G136" s="113">
         <v>0</v>
       </c>
-      <c r="H136" s="102">
+      <c r="H136" s="89">
         <v>0</v>
       </c>
-      <c r="I136" s="103">
+      <c r="I136" s="102">
         <v>0</v>
       </c>
-      <c r="J136" s="103">
+      <c r="J136" s="102">
         <v>0</v>
       </c>
     </row>
     <row r="137" spans="1:10">
-      <c r="A137" s="120" t="s">
+      <c r="A137" t="s">
         <v>7</v>
       </c>
-      <c r="B137" s="120" t="s">
+      <c r="B137" t="s">
         <v>2</v>
       </c>
-      <c r="C137" s="121" t="s">
+      <c r="C137" s="112" t="s">
         <v>132</v>
       </c>
-      <c r="D137" s="120" t="s">
+      <c r="D137" t="s">
         <v>218</v>
       </c>
-      <c r="E137" s="120" t="s">
+      <c r="E137" t="s">
         <v>192</v>
       </c>
-      <c r="F137" s="121" t="s">
+      <c r="F137" s="112" t="s">
         <v>752</v>
       </c>
-      <c r="G137" s="122">
+      <c r="G137" s="113">
         <v>0</v>
       </c>
-      <c r="H137" s="102">
+      <c r="H137" s="89">
         <v>0</v>
       </c>
-      <c r="I137" s="103">
+      <c r="I137" s="102">
         <v>0</v>
       </c>
-      <c r="J137" s="103">
+      <c r="J137" s="102">
         <v>0</v>
       </c>
     </row>
     <row r="138" spans="1:10">
-      <c r="A138" s="120" t="s">
+      <c r="A138" t="s">
         <v>7</v>
       </c>
-      <c r="B138" s="120" t="s">
+      <c r="B138" t="s">
         <v>2</v>
       </c>
-      <c r="C138" s="121" t="s">
+      <c r="C138" s="112" t="s">
         <v>132</v>
       </c>
-      <c r="D138" s="120" t="s">
+      <c r="D138" t="s">
         <v>219</v>
       </c>
-      <c r="E138" s="120" t="s">
+      <c r="E138" t="s">
         <v>192</v>
       </c>
-      <c r="F138" s="121" t="s">
+      <c r="F138" s="112" t="s">
         <v>752</v>
       </c>
-      <c r="G138" s="122">
+      <c r="G138" s="113">
         <v>0</v>
       </c>
-      <c r="H138" s="102">
+      <c r="H138" s="89">
         <v>0</v>
       </c>
-      <c r="I138" s="103">
+      <c r="I138" s="102">
         <v>0</v>
       </c>
-      <c r="J138" s="103">
+      <c r="J138" s="102">
         <v>0</v>
       </c>
     </row>
@@ -12541,7 +12533,7 @@
       <c r="B139" s="88" t="s">
         <v>2</v>
       </c>
-      <c r="C139" s="119" t="s">
+      <c r="C139" s="117" t="s">
         <v>132</v>
       </c>
       <c r="D139" s="88" t="s">
@@ -12550,19 +12542,19 @@
       <c r="E139" s="88" t="s">
         <v>334</v>
       </c>
-      <c r="F139" s="119" t="s">
+      <c r="F139" s="117" t="s">
         <v>757</v>
       </c>
-      <c r="G139" s="117">
+      <c r="G139" s="115">
         <v>0</v>
       </c>
-      <c r="H139" s="116">
+      <c r="H139" s="114">
         <v>0</v>
       </c>
-      <c r="I139" s="112">
+      <c r="I139" s="110">
         <v>0</v>
       </c>
-      <c r="J139" s="112">
+      <c r="J139" s="110">
         <v>0</v>
       </c>
     </row>

</xml_diff>